<commit_message>
chore(design): CI policy, kickoff, Slice 0 ledger ruling
</commit_message>
<xml_diff>
--- a/redesign/L0_ledger.xlsx
+++ b/redesign/L0_ledger.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,8 +61,13 @@
       <color rgb="001F3864"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -82,6 +87,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -111,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -126,6 +136,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -835,11 +848,19 @@
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="4" t="inlineStr"/>
-      <c r="J8" s="3" t="inlineStr"/>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>migrate</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Slice 0 · d0 leaf · → L0 foundation/money (Currency backing the Money type)</t>
+        </is>
+      </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>in quarry</t>
+          <t>in quarry (ruled — Slice 0)</t>
         </is>
       </c>
     </row>
@@ -972,11 +993,19 @@
           <t>type:ignore</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr"/>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>migrate</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Slice 0 · d0 leaf · → L0 foundation/time (year_fraction; Money at boundary)</t>
+        </is>
+      </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>in quarry</t>
+          <t>in quarry (ruled — Slice 0)</t>
         </is>
       </c>
     </row>
@@ -1058,11 +1087,19 @@
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="4" t="inlineStr"/>
-      <c r="J13" s="3" t="inlineStr"/>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>re-home</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Slice 0 · d1 · → L1 market: MINIMAL flat curve behind CurveHandle (df=exp(-r·t)); full curve at S2</t>
+        </is>
+      </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>in quarry</t>
+          <t>in quarry (ruled — Slice 0)</t>
         </is>
       </c>
     </row>
@@ -1402,11 +1439,19 @@
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr"/>
-      <c r="I21" s="4" t="inlineStr"/>
-      <c r="J21" s="3" t="inlineStr"/>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>migrate</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Slice 0 · d0 leaf · → L0 (explicit NumericalConfig; already frozen — pin it)</t>
+        </is>
+      </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>in quarry</t>
+          <t>in quarry (ruled — Slice 0)</t>
         </is>
       </c>
     </row>

</xml_diff>